<commit_message>
Stage 8 review fixes: A-015
</commit_message>
<xml_diff>
--- a/output/archive/Archive/Users/cantoine_old_laptop/Projects/FT09/FT09_analogue-delivery_30Mar16.xlsx
+++ b/output/archive/Archive/Users/cantoine_old_laptop/Projects/FT09/FT09_analogue-delivery_30Mar16.xlsx
@@ -175,12 +175,12 @@
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
-        <t>Lot list is the one from the shared drive, this copy is a month older. Use the shared one.</t>
+        <t>Keep the final delivery list with the assignment cards on the shared drive; this is my retained working copy.</t>
       </text>
     </comment>
     <comment ref="D5" authorId="1" shapeId="0">
       <text>
-        <t>Yield column came from the old template, check it matches the final cards before anyone quotes it.</t>
+        <t>Quote isolated yields with the final compound cards so the preparation basis stays clear.</t>
       </text>
     </comment>
   </commentList>
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -570,19 +570,19 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Delivered. Positional assignments in the N-substitution sheet are the ones we sent. The two open ones are flagged in the comments.</t>
+          <t>Delivered with positional assignments. Consult the final compound cards for the N-substitution map; this sheet does not reproduce the assignment evidence.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Chase</t>
+          <t>Filing note</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CA: NOESY for the N2 set is in the folder, not yet on the LIMS. Ask CF whether it goes in the lot record.</t>
+          <t>CA: keep the assignment spectra with the final compound cards so CF can find them with the lot record.</t>
         </is>
       </c>
     </row>
@@ -602,6 +602,18 @@
       <c r="D12" s="2" t="inlineStr">
         <is>
           <t>30/03/2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Vellacombe Discovery Ltd</t>
         </is>
       </c>
     </row>
@@ -620,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -638,115 +650,50 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Conditions</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Scale (mmol)</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Chemistry note</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N-substitution map</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>NaH, DMF, 0 C then alkyl bromide</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>0.5 per analogue</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Gives a mixture. Ratio is the thing to watch, so run both isomers through the column.</t>
+          <t>Positional assignments accompanied the completed delivery; refer to the final compound cards for each analogue.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Assignment evidence</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Cs2CO3, MeCN, 60 C</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>0.5 per analogue</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Favours N1 for the bulkier halides. Less useful for the small alkyls.</t>
+          <t>Keep the structure assignment and supporting spectra together. Do not assign indazole substitution position from a single overlapping proton shift.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Biology comparison</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Mitsunobu, DIAD, PPh3, THF</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>0.2 per analogue</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Only for the hydroxyethyl side chains. Slow but clean.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>N1 vs N2 by HMBC and NOESY. Not from 1H shifts alone, the shifts overlap on the aryl ring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Trend</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Two divergent potency trends. Seems to follow the N-substituent size, which is what the study plan asked for.</t>
+          <t>The positional assignments allow Feldorune to distinguish divergent potency trends. No potency results or substituent-size relationship are reported in this workbook.</t>
         </is>
       </c>
     </row>
@@ -784,7 +731,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yield is isolated. Purity is HPLC area % at 254 nm. Amounts are delivered mg per compound. Some SMILES here were typed in from the lab book and need checking.</t>
+          <t>Yield is isolated. Purity is HPLC area % at 254 nm. Amounts are delivered mg per compound. For positional assignments use the final compound cards.</t>
         </is>
       </c>
     </row>
@@ -1839,14 +1786,14 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>todo: send NOESY to CF</t>
+          <t>filing: keep assignment spectra with CF release records</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>todo: redo the Mitsunobu for FT09-07015 if the lot is short</t>
+          <t>filing: use the final compound card for any repeat preparation</t>
         </is>
       </c>
     </row>

</xml_diff>